<commit_message>
Remove example rows from feedback Excel template
</commit_message>
<xml_diff>
--- a/novustruck-homepage-feedback.xlsx
+++ b/novustruck-homepage-feedback.xlsx
@@ -105,7 +105,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -127,11 +127,55 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -184,6 +228,8 @@
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -613,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -675,107 +721,49 @@
           <t>👉  Fülle bitte für jeden Punkt eine eigene Zeile aus. Bereich aus der Dropdown-Liste wählen.</t>
         </is>
       </c>
+      <c r="B3" s="18" t="n"/>
+      <c r="C3" s="18" t="n"/>
+      <c r="D3" s="18" t="n"/>
+      <c r="E3" s="18" t="n"/>
+      <c r="F3" s="18" t="n"/>
+      <c r="G3" s="19" t="n"/>
     </row>
     <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="4" t="n">
+      <c r="A4" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Navigation</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Logo zu klein auf Mobile</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>Logo größer / andere Farbe</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Mittel</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Offen</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>Auf iPhone 14 kaum sichtbar</t>
-        </is>
-      </c>
+      <c r="B4" s="12" t="n"/>
+      <c r="C4" s="12" t="n"/>
+      <c r="D4" s="12" t="n"/>
+      <c r="E4" s="13" t="n"/>
+      <c r="F4" s="13" t="n"/>
+      <c r="G4" s="12" t="n"/>
     </row>
     <row r="5" ht="28" customHeight="1">
-      <c r="A5" s="6" t="n">
+      <c r="A5" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>Video</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Video startet nicht sofort</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>Sofort abspielen ohne Klick</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>Hoch</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>Offen</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr"/>
+      <c r="B5" s="9" t="n"/>
+      <c r="C5" s="9" t="n"/>
+      <c r="D5" s="9" t="n"/>
+      <c r="E5" s="10" t="n"/>
+      <c r="F5" s="10" t="n"/>
+      <c r="G5" s="9" t="n"/>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="4" t="n">
+      <c r="A6" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>News</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Zu wenig News-Beiträge auf der Seite</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>3. Newscard mit neuem Bericht</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Niedrig</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Offen</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr"/>
+      <c r="B6" s="12" t="n"/>
+      <c r="C6" s="12" t="n"/>
+      <c r="D6" s="12" t="n"/>
+      <c r="E6" s="13" t="n"/>
+      <c r="F6" s="13" t="n"/>
+      <c r="G6" s="12" t="n"/>
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B7" s="9" t="n"/>
       <c r="C7" s="9" t="n"/>
@@ -786,7 +774,7 @@
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="11" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B8" s="12" t="n"/>
       <c r="C8" s="12" t="n"/>
@@ -797,7 +785,7 @@
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="8" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B9" s="9" t="n"/>
       <c r="C9" s="9" t="n"/>
@@ -808,7 +796,7 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="11" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B10" s="12" t="n"/>
       <c r="C10" s="12" t="n"/>
@@ -819,7 +807,7 @@
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="8" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B11" s="9" t="n"/>
       <c r="C11" s="9" t="n"/>
@@ -830,7 +818,7 @@
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="11" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B12" s="12" t="n"/>
       <c r="C12" s="12" t="n"/>
@@ -841,7 +829,7 @@
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="8" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B13" s="9" t="n"/>
       <c r="C13" s="9" t="n"/>
@@ -852,7 +840,7 @@
     </row>
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="11" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B14" s="12" t="n"/>
       <c r="C14" s="12" t="n"/>
@@ -863,7 +851,7 @@
     </row>
     <row r="15" ht="28" customHeight="1">
       <c r="A15" s="8" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B15" s="9" t="n"/>
       <c r="C15" s="9" t="n"/>
@@ -874,7 +862,7 @@
     </row>
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="11" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B16" s="12" t="n"/>
       <c r="C16" s="12" t="n"/>
@@ -885,7 +873,7 @@
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="8" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B17" s="9" t="n"/>
       <c r="C17" s="9" t="n"/>
@@ -896,7 +884,7 @@
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="11" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B18" s="12" t="n"/>
       <c r="C18" s="12" t="n"/>
@@ -907,7 +895,7 @@
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="8" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B19" s="9" t="n"/>
       <c r="C19" s="9" t="n"/>
@@ -918,7 +906,7 @@
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="11" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B20" s="12" t="n"/>
       <c r="C20" s="12" t="n"/>
@@ -929,7 +917,7 @@
     </row>
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="8" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B21" s="9" t="n"/>
       <c r="C21" s="9" t="n"/>
@@ -940,7 +928,7 @@
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="11" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B22" s="12" t="n"/>
       <c r="C22" s="12" t="n"/>
@@ -951,7 +939,7 @@
     </row>
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="8" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B23" s="9" t="n"/>
       <c r="C23" s="9" t="n"/>
@@ -962,7 +950,7 @@
     </row>
     <row r="24" ht="28" customHeight="1">
       <c r="A24" s="11" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B24" s="12" t="n"/>
       <c r="C24" s="12" t="n"/>
@@ -973,7 +961,7 @@
     </row>
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="8" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B25" s="9" t="n"/>
       <c r="C25" s="9" t="n"/>
@@ -984,7 +972,7 @@
     </row>
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="11" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B26" s="12" t="n"/>
       <c r="C26" s="12" t="n"/>
@@ -995,7 +983,7 @@
     </row>
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="8" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B27" s="9" t="n"/>
       <c r="C27" s="9" t="n"/>
@@ -1006,7 +994,7 @@
     </row>
     <row r="28" ht="28" customHeight="1">
       <c r="A28" s="11" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B28" s="12" t="n"/>
       <c r="C28" s="12" t="n"/>
@@ -1017,7 +1005,7 @@
     </row>
     <row r="29" ht="28" customHeight="1">
       <c r="A29" s="8" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B29" s="9" t="n"/>
       <c r="C29" s="9" t="n"/>
@@ -1028,7 +1016,7 @@
     </row>
     <row r="30" ht="28" customHeight="1">
       <c r="A30" s="11" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B30" s="12" t="n"/>
       <c r="C30" s="12" t="n"/>
@@ -1039,7 +1027,7 @@
     </row>
     <row r="31" ht="28" customHeight="1">
       <c r="A31" s="8" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B31" s="9" t="n"/>
       <c r="C31" s="9" t="n"/>
@@ -1050,7 +1038,7 @@
     </row>
     <row r="32" ht="28" customHeight="1">
       <c r="A32" s="11" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B32" s="12" t="n"/>
       <c r="C32" s="12" t="n"/>
@@ -1061,7 +1049,7 @@
     </row>
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="8" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B33" s="9" t="n"/>
       <c r="C33" s="9" t="n"/>
@@ -1070,39 +1058,9 @@
       <c r="F33" s="10" t="n"/>
       <c r="G33" s="9" t="n"/>
     </row>
-    <row r="34" ht="28" customHeight="1">
-      <c r="A34" s="11" t="n">
-        <v>28</v>
-      </c>
-      <c r="B34" s="12" t="n"/>
-      <c r="C34" s="12" t="n"/>
-      <c r="D34" s="12" t="n"/>
-      <c r="E34" s="13" t="n"/>
-      <c r="F34" s="13" t="n"/>
-      <c r="G34" s="12" t="n"/>
-    </row>
-    <row r="35" ht="28" customHeight="1">
-      <c r="A35" s="8" t="n">
-        <v>29</v>
-      </c>
-      <c r="B35" s="9" t="n"/>
-      <c r="C35" s="9" t="n"/>
-      <c r="D35" s="9" t="n"/>
-      <c r="E35" s="10" t="n"/>
-      <c r="F35" s="10" t="n"/>
-      <c r="G35" s="9" t="n"/>
-    </row>
-    <row r="36" ht="28" customHeight="1">
-      <c r="A36" s="11" t="n">
-        <v>30</v>
-      </c>
-      <c r="B36" s="12" t="n"/>
-      <c r="C36" s="12" t="n"/>
-      <c r="D36" s="12" t="n"/>
-      <c r="E36" s="13" t="n"/>
-      <c r="F36" s="13" t="n"/>
-      <c r="G36" s="12" t="n"/>
-    </row>
+    <row r="34" ht="28" customHeight="1"/>
+    <row r="35" ht="28" customHeight="1"/>
+    <row r="36" ht="28" customHeight="1"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A3:G3"/>

</xml_diff>

<commit_message>
Translate feedback Excel template to English
</commit_message>
<xml_diff>
--- a/novustruck-homepage-feedback.xlsx
+++ b/novustruck-homepage-feedback.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Feedback Homepage" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Bereiche &amp; Legende" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Homepage Feedback" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sections &amp; Legend" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,12 +42,6 @@
       <name val="Calibri"/>
       <i val="1"/>
       <color rgb="007A6A00"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="00555555"/>
       <sz val="9"/>
     </font>
     <font>
@@ -105,7 +99,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -127,55 +121,11 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00CCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00CCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -186,50 +136,36 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -674,34 +610,34 @@
     <row r="1" ht="14" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>NOVUS automotive group — Homepage Feedback &amp; Verbesserungswünsche</t>
+          <t>NOVUS automotive group — Homepage Feedback &amp; Improvement Requests</t>
         </is>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Nr.</t>
+          <t>No.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Bereich</t>
+          <t>Section</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Was gefällt nicht / Fehler</t>
+          <t>Issue / What doesn't work</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Verbesserungswunsch</t>
+          <t>Improvement Request</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Priorität</t>
+          <t>Priority</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -711,389 +647,380 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Notizen / Details</t>
+          <t>Notes / Details</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>👉  Fülle bitte für jeden Punkt eine eigene Zeile aus. Bereich aus der Dropdown-Liste wählen.</t>
-        </is>
-      </c>
-      <c r="B3" s="18" t="n"/>
-      <c r="C3" s="18" t="n"/>
-      <c r="D3" s="18" t="n"/>
-      <c r="E3" s="18" t="n"/>
-      <c r="F3" s="18" t="n"/>
-      <c r="G3" s="19" t="n"/>
+          <t>👉  Please fill in one row per issue. Select section from the dropdown list.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="11" t="n">
+      <c r="A4" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="12" t="n"/>
-      <c r="C4" s="12" t="n"/>
-      <c r="D4" s="12" t="n"/>
-      <c r="E4" s="13" t="n"/>
-      <c r="F4" s="13" t="n"/>
-      <c r="G4" s="12" t="n"/>
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="5" t="n"/>
     </row>
     <row r="5" ht="28" customHeight="1">
-      <c r="A5" s="8" t="n">
+      <c r="A5" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="9" t="n"/>
-      <c r="C5" s="9" t="n"/>
-      <c r="D5" s="9" t="n"/>
-      <c r="E5" s="10" t="n"/>
-      <c r="F5" s="10" t="n"/>
-      <c r="G5" s="9" t="n"/>
+      <c r="B5" s="8" t="n"/>
+      <c r="C5" s="8" t="n"/>
+      <c r="D5" s="8" t="n"/>
+      <c r="E5" s="9" t="n"/>
+      <c r="F5" s="9" t="n"/>
+      <c r="G5" s="8" t="n"/>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="11" t="n">
+      <c r="A6" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="12" t="n"/>
-      <c r="C6" s="12" t="n"/>
-      <c r="D6" s="12" t="n"/>
-      <c r="E6" s="13" t="n"/>
-      <c r="F6" s="13" t="n"/>
-      <c r="G6" s="12" t="n"/>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="5" t="n"/>
     </row>
     <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="8" t="n">
+      <c r="A7" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="9" t="n"/>
-      <c r="C7" s="9" t="n"/>
-      <c r="D7" s="9" t="n"/>
-      <c r="E7" s="10" t="n"/>
-      <c r="F7" s="10" t="n"/>
-      <c r="G7" s="9" t="n"/>
+      <c r="B7" s="8" t="n"/>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="8" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n"/>
+      <c r="G7" s="8" t="n"/>
     </row>
     <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="11" t="n">
+      <c r="A8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="12" t="n"/>
-      <c r="C8" s="12" t="n"/>
-      <c r="D8" s="12" t="n"/>
-      <c r="E8" s="13" t="n"/>
-      <c r="F8" s="13" t="n"/>
-      <c r="G8" s="12" t="n"/>
+      <c r="B8" s="5" t="n"/>
+      <c r="C8" s="5" t="n"/>
+      <c r="D8" s="5" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="5" t="n"/>
     </row>
     <row r="9" ht="28" customHeight="1">
-      <c r="A9" s="8" t="n">
+      <c r="A9" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="9" t="n"/>
-      <c r="C9" s="9" t="n"/>
-      <c r="D9" s="9" t="n"/>
-      <c r="E9" s="10" t="n"/>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="9" t="n"/>
+      <c r="B9" s="8" t="n"/>
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="8" t="n"/>
+      <c r="E9" s="9" t="n"/>
+      <c r="F9" s="9" t="n"/>
+      <c r="G9" s="8" t="n"/>
     </row>
     <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="11" t="n">
+      <c r="A10" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="12" t="n"/>
-      <c r="C10" s="12" t="n"/>
-      <c r="D10" s="12" t="n"/>
-      <c r="E10" s="13" t="n"/>
-      <c r="F10" s="13" t="n"/>
-      <c r="G10" s="12" t="n"/>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="5" t="n"/>
     </row>
     <row r="11" ht="28" customHeight="1">
-      <c r="A11" s="8" t="n">
+      <c r="A11" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="9" t="n"/>
-      <c r="C11" s="9" t="n"/>
-      <c r="D11" s="9" t="n"/>
-      <c r="E11" s="10" t="n"/>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="9" t="n"/>
+      <c r="B11" s="8" t="n"/>
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="8" t="n"/>
+      <c r="E11" s="9" t="n"/>
+      <c r="F11" s="9" t="n"/>
+      <c r="G11" s="8" t="n"/>
     </row>
     <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="11" t="n">
+      <c r="A12" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="12" t="n"/>
-      <c r="C12" s="12" t="n"/>
-      <c r="D12" s="12" t="n"/>
-      <c r="E12" s="13" t="n"/>
-      <c r="F12" s="13" t="n"/>
-      <c r="G12" s="12" t="n"/>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="5" t="n"/>
     </row>
     <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="8" t="n">
+      <c r="A13" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="9" t="n"/>
-      <c r="C13" s="9" t="n"/>
-      <c r="D13" s="9" t="n"/>
-      <c r="E13" s="10" t="n"/>
-      <c r="F13" s="10" t="n"/>
-      <c r="G13" s="9" t="n"/>
+      <c r="B13" s="8" t="n"/>
+      <c r="C13" s="8" t="n"/>
+      <c r="D13" s="8" t="n"/>
+      <c r="E13" s="9" t="n"/>
+      <c r="F13" s="9" t="n"/>
+      <c r="G13" s="8" t="n"/>
     </row>
     <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="11" t="n">
+      <c r="A14" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="12" t="n"/>
-      <c r="C14" s="12" t="n"/>
-      <c r="D14" s="12" t="n"/>
-      <c r="E14" s="13" t="n"/>
-      <c r="F14" s="13" t="n"/>
-      <c r="G14" s="12" t="n"/>
+      <c r="B14" s="5" t="n"/>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="5" t="n"/>
     </row>
     <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="8" t="n">
+      <c r="A15" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="9" t="n"/>
-      <c r="C15" s="9" t="n"/>
-      <c r="D15" s="9" t="n"/>
-      <c r="E15" s="10" t="n"/>
-      <c r="F15" s="10" t="n"/>
-      <c r="G15" s="9" t="n"/>
+      <c r="B15" s="8" t="n"/>
+      <c r="C15" s="8" t="n"/>
+      <c r="D15" s="8" t="n"/>
+      <c r="E15" s="9" t="n"/>
+      <c r="F15" s="9" t="n"/>
+      <c r="G15" s="8" t="n"/>
     </row>
     <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="11" t="n">
+      <c r="A16" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="12" t="n"/>
-      <c r="C16" s="12" t="n"/>
-      <c r="D16" s="12" t="n"/>
-      <c r="E16" s="13" t="n"/>
-      <c r="F16" s="13" t="n"/>
-      <c r="G16" s="12" t="n"/>
+      <c r="B16" s="5" t="n"/>
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="5" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="5" t="n"/>
     </row>
     <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="8" t="n">
+      <c r="A17" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="9" t="n"/>
-      <c r="C17" s="9" t="n"/>
-      <c r="D17" s="9" t="n"/>
-      <c r="E17" s="10" t="n"/>
-      <c r="F17" s="10" t="n"/>
-      <c r="G17" s="9" t="n"/>
+      <c r="B17" s="8" t="n"/>
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="8" t="n"/>
+      <c r="E17" s="9" t="n"/>
+      <c r="F17" s="9" t="n"/>
+      <c r="G17" s="8" t="n"/>
     </row>
     <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="11" t="n">
+      <c r="A18" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="12" t="n"/>
-      <c r="C18" s="12" t="n"/>
-      <c r="D18" s="12" t="n"/>
-      <c r="E18" s="13" t="n"/>
-      <c r="F18" s="13" t="n"/>
-      <c r="G18" s="12" t="n"/>
+      <c r="B18" s="5" t="n"/>
+      <c r="C18" s="5" t="n"/>
+      <c r="D18" s="5" t="n"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="5" t="n"/>
     </row>
     <row r="19" ht="28" customHeight="1">
-      <c r="A19" s="8" t="n">
+      <c r="A19" s="7" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="9" t="n"/>
-      <c r="C19" s="9" t="n"/>
-      <c r="D19" s="9" t="n"/>
-      <c r="E19" s="10" t="n"/>
-      <c r="F19" s="10" t="n"/>
-      <c r="G19" s="9" t="n"/>
+      <c r="B19" s="8" t="n"/>
+      <c r="C19" s="8" t="n"/>
+      <c r="D19" s="8" t="n"/>
+      <c r="E19" s="9" t="n"/>
+      <c r="F19" s="9" t="n"/>
+      <c r="G19" s="8" t="n"/>
     </row>
     <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="11" t="n">
+      <c r="A20" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="B20" s="12" t="n"/>
-      <c r="C20" s="12" t="n"/>
-      <c r="D20" s="12" t="n"/>
-      <c r="E20" s="13" t="n"/>
-      <c r="F20" s="13" t="n"/>
-      <c r="G20" s="12" t="n"/>
+      <c r="B20" s="5" t="n"/>
+      <c r="C20" s="5" t="n"/>
+      <c r="D20" s="5" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="5" t="n"/>
     </row>
     <row r="21" ht="28" customHeight="1">
-      <c r="A21" s="8" t="n">
+      <c r="A21" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="9" t="n"/>
-      <c r="C21" s="9" t="n"/>
-      <c r="D21" s="9" t="n"/>
-      <c r="E21" s="10" t="n"/>
-      <c r="F21" s="10" t="n"/>
-      <c r="G21" s="9" t="n"/>
+      <c r="B21" s="8" t="n"/>
+      <c r="C21" s="8" t="n"/>
+      <c r="D21" s="8" t="n"/>
+      <c r="E21" s="9" t="n"/>
+      <c r="F21" s="9" t="n"/>
+      <c r="G21" s="8" t="n"/>
     </row>
     <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="11" t="n">
+      <c r="A22" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="B22" s="12" t="n"/>
-      <c r="C22" s="12" t="n"/>
-      <c r="D22" s="12" t="n"/>
-      <c r="E22" s="13" t="n"/>
-      <c r="F22" s="13" t="n"/>
-      <c r="G22" s="12" t="n"/>
+      <c r="B22" s="5" t="n"/>
+      <c r="C22" s="5" t="n"/>
+      <c r="D22" s="5" t="n"/>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="n"/>
+      <c r="G22" s="5" t="n"/>
     </row>
     <row r="23" ht="28" customHeight="1">
-      <c r="A23" s="8" t="n">
+      <c r="A23" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="B23" s="9" t="n"/>
-      <c r="C23" s="9" t="n"/>
-      <c r="D23" s="9" t="n"/>
-      <c r="E23" s="10" t="n"/>
-      <c r="F23" s="10" t="n"/>
-      <c r="G23" s="9" t="n"/>
+      <c r="B23" s="8" t="n"/>
+      <c r="C23" s="8" t="n"/>
+      <c r="D23" s="8" t="n"/>
+      <c r="E23" s="9" t="n"/>
+      <c r="F23" s="9" t="n"/>
+      <c r="G23" s="8" t="n"/>
     </row>
     <row r="24" ht="28" customHeight="1">
-      <c r="A24" s="11" t="n">
+      <c r="A24" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="B24" s="12" t="n"/>
-      <c r="C24" s="12" t="n"/>
-      <c r="D24" s="12" t="n"/>
-      <c r="E24" s="13" t="n"/>
-      <c r="F24" s="13" t="n"/>
-      <c r="G24" s="12" t="n"/>
+      <c r="B24" s="5" t="n"/>
+      <c r="C24" s="5" t="n"/>
+      <c r="D24" s="5" t="n"/>
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="6" t="n"/>
+      <c r="G24" s="5" t="n"/>
     </row>
     <row r="25" ht="28" customHeight="1">
-      <c r="A25" s="8" t="n">
+      <c r="A25" s="7" t="n">
         <v>22</v>
       </c>
-      <c r="B25" s="9" t="n"/>
-      <c r="C25" s="9" t="n"/>
-      <c r="D25" s="9" t="n"/>
-      <c r="E25" s="10" t="n"/>
-      <c r="F25" s="10" t="n"/>
-      <c r="G25" s="9" t="n"/>
+      <c r="B25" s="8" t="n"/>
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="8" t="n"/>
+      <c r="E25" s="9" t="n"/>
+      <c r="F25" s="9" t="n"/>
+      <c r="G25" s="8" t="n"/>
     </row>
     <row r="26" ht="28" customHeight="1">
-      <c r="A26" s="11" t="n">
+      <c r="A26" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="B26" s="12" t="n"/>
-      <c r="C26" s="12" t="n"/>
-      <c r="D26" s="12" t="n"/>
-      <c r="E26" s="13" t="n"/>
-      <c r="F26" s="13" t="n"/>
-      <c r="G26" s="12" t="n"/>
+      <c r="B26" s="5" t="n"/>
+      <c r="C26" s="5" t="n"/>
+      <c r="D26" s="5" t="n"/>
+      <c r="E26" s="6" t="n"/>
+      <c r="F26" s="6" t="n"/>
+      <c r="G26" s="5" t="n"/>
     </row>
     <row r="27" ht="28" customHeight="1">
-      <c r="A27" s="8" t="n">
+      <c r="A27" s="7" t="n">
         <v>24</v>
       </c>
-      <c r="B27" s="9" t="n"/>
-      <c r="C27" s="9" t="n"/>
-      <c r="D27" s="9" t="n"/>
-      <c r="E27" s="10" t="n"/>
-      <c r="F27" s="10" t="n"/>
-      <c r="G27" s="9" t="n"/>
+      <c r="B27" s="8" t="n"/>
+      <c r="C27" s="8" t="n"/>
+      <c r="D27" s="8" t="n"/>
+      <c r="E27" s="9" t="n"/>
+      <c r="F27" s="9" t="n"/>
+      <c r="G27" s="8" t="n"/>
     </row>
     <row r="28" ht="28" customHeight="1">
-      <c r="A28" s="11" t="n">
+      <c r="A28" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="B28" s="12" t="n"/>
-      <c r="C28" s="12" t="n"/>
-      <c r="D28" s="12" t="n"/>
-      <c r="E28" s="13" t="n"/>
-      <c r="F28" s="13" t="n"/>
-      <c r="G28" s="12" t="n"/>
+      <c r="B28" s="5" t="n"/>
+      <c r="C28" s="5" t="n"/>
+      <c r="D28" s="5" t="n"/>
+      <c r="E28" s="6" t="n"/>
+      <c r="F28" s="6" t="n"/>
+      <c r="G28" s="5" t="n"/>
     </row>
     <row r="29" ht="28" customHeight="1">
-      <c r="A29" s="8" t="n">
+      <c r="A29" s="7" t="n">
         <v>26</v>
       </c>
-      <c r="B29" s="9" t="n"/>
-      <c r="C29" s="9" t="n"/>
-      <c r="D29" s="9" t="n"/>
-      <c r="E29" s="10" t="n"/>
-      <c r="F29" s="10" t="n"/>
-      <c r="G29" s="9" t="n"/>
+      <c r="B29" s="8" t="n"/>
+      <c r="C29" s="8" t="n"/>
+      <c r="D29" s="8" t="n"/>
+      <c r="E29" s="9" t="n"/>
+      <c r="F29" s="9" t="n"/>
+      <c r="G29" s="8" t="n"/>
     </row>
     <row r="30" ht="28" customHeight="1">
-      <c r="A30" s="11" t="n">
+      <c r="A30" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="B30" s="12" t="n"/>
-      <c r="C30" s="12" t="n"/>
-      <c r="D30" s="12" t="n"/>
-      <c r="E30" s="13" t="n"/>
-      <c r="F30" s="13" t="n"/>
-      <c r="G30" s="12" t="n"/>
+      <c r="B30" s="5" t="n"/>
+      <c r="C30" s="5" t="n"/>
+      <c r="D30" s="5" t="n"/>
+      <c r="E30" s="6" t="n"/>
+      <c r="F30" s="6" t="n"/>
+      <c r="G30" s="5" t="n"/>
     </row>
     <row r="31" ht="28" customHeight="1">
-      <c r="A31" s="8" t="n">
+      <c r="A31" s="7" t="n">
         <v>28</v>
       </c>
-      <c r="B31" s="9" t="n"/>
-      <c r="C31" s="9" t="n"/>
-      <c r="D31" s="9" t="n"/>
-      <c r="E31" s="10" t="n"/>
-      <c r="F31" s="10" t="n"/>
-      <c r="G31" s="9" t="n"/>
+      <c r="B31" s="8" t="n"/>
+      <c r="C31" s="8" t="n"/>
+      <c r="D31" s="8" t="n"/>
+      <c r="E31" s="9" t="n"/>
+      <c r="F31" s="9" t="n"/>
+      <c r="G31" s="8" t="n"/>
     </row>
     <row r="32" ht="28" customHeight="1">
-      <c r="A32" s="11" t="n">
+      <c r="A32" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="B32" s="12" t="n"/>
-      <c r="C32" s="12" t="n"/>
-      <c r="D32" s="12" t="n"/>
-      <c r="E32" s="13" t="n"/>
-      <c r="F32" s="13" t="n"/>
-      <c r="G32" s="12" t="n"/>
+      <c r="B32" s="5" t="n"/>
+      <c r="C32" s="5" t="n"/>
+      <c r="D32" s="5" t="n"/>
+      <c r="E32" s="6" t="n"/>
+      <c r="F32" s="6" t="n"/>
+      <c r="G32" s="5" t="n"/>
     </row>
     <row r="33" ht="28" customHeight="1">
-      <c r="A33" s="8" t="n">
+      <c r="A33" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="B33" s="9" t="n"/>
-      <c r="C33" s="9" t="n"/>
-      <c r="D33" s="9" t="n"/>
-      <c r="E33" s="10" t="n"/>
-      <c r="F33" s="10" t="n"/>
-      <c r="G33" s="9" t="n"/>
-    </row>
-    <row r="34" ht="28" customHeight="1"/>
-    <row r="35" ht="28" customHeight="1"/>
-    <row r="36" ht="28" customHeight="1"/>
+      <c r="B33" s="8" t="n"/>
+      <c r="C33" s="8" t="n"/>
+      <c r="D33" s="8" t="n"/>
+      <c r="E33" s="9" t="n"/>
+      <c r="F33" s="9" t="n"/>
+      <c r="G33" s="8" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A3:G3"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <conditionalFormatting sqref="E4:E36">
+  <conditionalFormatting sqref="E4:E33">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>"Hoch"</formula>
+      <formula>"High"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
-      <formula>"Mittel"</formula>
+      <formula>"Medium"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
-      <formula>"Niedrig"</formula>
+      <formula>"Low"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F4:F36">
+  <conditionalFormatting sqref="F4:F33">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
-      <formula>"Erledigt"</formula>
+      <formula>"Done"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
-      <formula>"In Arbeit"</formula>
+      <formula>"In Progress"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="B4:B36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültiger Bereich" error="Bitte aus der Liste wählen" type="list">
-      <formula1>"Navigation,Hero/Banner,Video,News,Modelle,Technik,Händler-Karte,Kontakt,Footer,Impressum,Datenschutz,Mobile/Tablet,Allgemein"</formula1>
+    <dataValidation sqref="B4:B33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Navigation,Hero/Banner,Video,News,Models,Technology,Dealer Map,Contact,Footer,Legal Notice,Privacy Policy,Mobile/Tablet,General"</formula1>
     </dataValidation>
-    <dataValidation sqref="E4:E36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Hoch,Mittel,Niedrig"</formula1>
+    <dataValidation sqref="E4:E33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation sqref="F4:F36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Offen,In Arbeit,Erledigt"</formula1>
+    <dataValidation sqref="F4:F33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Open,In Progress,Done"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1111,181 +1038,181 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="14" t="inlineStr">
-        <is>
-          <t>Bereiche der Homepage — Erklärung</t>
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Homepage Sections — Description</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
-        <is>
-          <t>Bereich</t>
-        </is>
-      </c>
-      <c r="B2" s="15" t="inlineStr">
-        <is>
-          <t>Beschreibung</t>
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>Description</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="16" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Navigation</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
-        <is>
-          <t>Menü oben (Logo, Links, Kontakt-Button)</t>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>Top menu bar (logo, links, contact button)</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>Hero/Banner</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
-        <is>
-          <t>Großes Bild/Text ganz oben auf der Startseite</t>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Large image/text at the very top of the homepage</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Video</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>Hintergrundvideo-Bereich mit SITRAK</t>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>Background video section with SITRAK truck</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>News</t>
         </is>
       </c>
-      <c r="B6" s="17" t="inlineStr">
-        <is>
-          <t>News-Karten-Bereich (3 Karten)</t>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>News card section (3 cards)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
-        <is>
-          <t>Modelle</t>
-        </is>
-      </c>
-      <c r="B7" s="16" t="inlineStr">
-        <is>
-          <t>LKW-Modell-Sektion (C7H, 4×2 etc.)</t>
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Models</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>Truck model section (C7H, 4×2, etc.)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="17" t="inlineStr">
-        <is>
-          <t>Technik</t>
-        </is>
-      </c>
-      <c r="B8" s="17" t="inlineStr">
-        <is>
-          <t>Features / Technik-Highlights-Sektion</t>
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Features / Technology highlights section</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="16" t="inlineStr">
-        <is>
-          <t>Händler-Karte</t>
-        </is>
-      </c>
-      <c r="B9" s="16" t="inlineStr">
-        <is>
-          <t>Karte mit Händler &amp; Service-Partnern</t>
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Dealer Map</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Map with dealers &amp; service partners</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="17" t="inlineStr">
-        <is>
-          <t>Kontakt</t>
-        </is>
-      </c>
-      <c r="B10" s="17" t="inlineStr">
-        <is>
-          <t>Kontaktformular-Bereich</t>
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Contact form section</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>Footer</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
-        <is>
-          <t>Fußzeile der Seite</t>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Bottom footer of the page</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="17" t="inlineStr">
-        <is>
-          <t>Impressum</t>
-        </is>
-      </c>
-      <c r="B12" s="17" t="inlineStr">
-        <is>
-          <t>Impressum-Seite (eigene Seite)</t>
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Legal Notice</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Legal notice page (separate page)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="16" t="inlineStr">
-        <is>
-          <t>Datenschutz</t>
-        </is>
-      </c>
-      <c r="B13" s="16" t="inlineStr">
-        <is>
-          <t>Datenschutz-Seite (eigene Seite)</t>
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>Privacy Policy</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>Privacy policy page (separate page)</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="A14" s="13" t="inlineStr">
         <is>
           <t>Mobile/Tablet</t>
         </is>
       </c>
-      <c r="B14" s="17" t="inlineStr">
-        <is>
-          <t>Darstellung auf Smartphone oder Tablet</t>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Display on smartphone or tablet</t>
         </is>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="16" t="inlineStr">
-        <is>
-          <t>Allgemein</t>
-        </is>
-      </c>
-      <c r="B15" s="16" t="inlineStr">
-        <is>
-          <t>Allgemeines Feedback, keinem Bereich zuzuordnen</t>
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>General feedback not tied to a specific section</t>
         </is>
       </c>
     </row>

</xml_diff>